<commit_message>
add wait buff dianguc
</commit_message>
<xml_diff>
--- a/Dianguc.xlsx
+++ b/Dianguc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tool\Xola\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Project\.tool\hiep\Xola\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E16A34D3-9D3B-472D-9F79-33BA612B3929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9B21AB-16AD-43FF-A441-B6295137C680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{210B81C1-063E-40AF-8D8C-307F53B87FDC}"/>
+    <workbookView xWindow="18984" yWindow="0" windowWidth="4152" windowHeight="13776" activeTab="3" xr2:uid="{210B81C1-063E-40AF-8D8C-307F53B87FDC}"/>
   </bookViews>
   <sheets>
     <sheet name="T3" sheetId="1" r:id="rId1"/>
@@ -19,22 +19,10 @@
     <sheet name="T6" sheetId="4" r:id="rId4"/>
     <sheet name="Sheet1" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -76,21 +64,28 @@
     <t>phải</t>
   </si>
   <si>
-    <t>sai</t>
+    <t>đúng</t>
   </si>
   <si>
-    <t>đúng</t>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -174,7 +169,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -183,6 +178,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -195,7 +191,8 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -511,22 +508,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4CB08FB-80B1-4D9C-AAE4-0416F8953E35}">
   <dimension ref="A1:I33"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="b">
+      <c r="C1" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -537,7 +534,7 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -548,7 +545,7 @@
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -559,7 +556,7 @@
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -570,7 +567,7 @@
       <c r="D5" s="3"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -581,7 +578,7 @@
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -592,7 +589,7 @@
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -603,7 +600,7 @@
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -614,7 +611,7 @@
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -625,7 +622,7 @@
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -636,7 +633,7 @@
       <c r="D11" s="3"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -649,7 +646,7 @@
       </c>
       <c r="E12" s="1"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -657,11 +654,11 @@
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -670,7 +667,7 @@
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -679,7 +676,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -688,7 +685,7 @@
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -697,7 +694,7 @@
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -706,7 +703,7 @@
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -715,7 +712,7 @@
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -724,7 +721,7 @@
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -733,7 +730,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -742,7 +739,7 @@
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -751,7 +748,7 @@
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -760,7 +757,7 @@
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -769,7 +766,7 @@
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -778,7 +775,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -787,7 +784,7 @@
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -796,7 +793,7 @@
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -805,7 +802,7 @@
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -814,7 +811,7 @@
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -823,8 +820,8 @@
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="8" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="9" t="s">
         <v>4</v>
       </c>
       <c r="B32" s="3" t="s">
@@ -840,8 +837,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="8"/>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="9"/>
       <c r="B33" s="1">
         <f>COUNTIF(B2:B31, "Up") / COUNTA(A2:A31)</f>
         <v>6.6666666666666666E-2</v>
@@ -872,22 +869,22 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{064059B2-0CFC-4C91-B4E1-43670BB0799C}">
   <dimension ref="A1:I43"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="b">
+      <c r="C1" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -898,7 +895,7 @@
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -909,7 +906,7 @@
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -920,7 +917,7 @@
       <c r="D4" s="5"/>
       <c r="E4" s="5"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -931,7 +928,7 @@
       <c r="D5" s="4"/>
       <c r="E5" s="5"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -942,7 +939,7 @@
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -953,7 +950,7 @@
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -964,7 +961,7 @@
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -975,7 +972,7 @@
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -986,7 +983,7 @@
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -997,7 +994,7 @@
       <c r="D11" s="4"/>
       <c r="E11" s="5"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1008,7 +1005,7 @@
       <c r="D12" s="4"/>
       <c r="E12" s="5"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1018,11 +1015,11 @@
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1033,7 +1030,7 @@
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1044,7 +1041,7 @@
       <c r="D15" s="3"/>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1055,7 +1052,7 @@
       <c r="D16" s="3"/>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -1066,7 +1063,7 @@
       <c r="D17" s="3"/>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1077,7 +1074,7 @@
       <c r="D18" s="3"/>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -1088,7 +1085,7 @@
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1099,7 +1096,7 @@
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1110,7 +1107,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -1121,7 +1118,7 @@
       <c r="D22" s="3"/>
       <c r="E22" s="3"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -1132,7 +1129,7 @@
       <c r="D23" s="3"/>
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -1143,7 +1140,7 @@
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -1154,7 +1151,7 @@
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -1165,7 +1162,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -1176,7 +1173,7 @@
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -1187,7 +1184,7 @@
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -1198,7 +1195,7 @@
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -1209,7 +1206,7 @@
       <c r="D30" s="3"/>
       <c r="E30" s="3"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -1220,7 +1217,7 @@
       <c r="D31" s="3"/>
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -1231,7 +1228,7 @@
       <c r="D32" s="3"/>
       <c r="E32" s="3"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -1242,7 +1239,7 @@
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -1253,7 +1250,7 @@
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -1264,7 +1261,7 @@
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -1275,7 +1272,7 @@
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -1286,7 +1283,7 @@
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -1297,7 +1294,7 @@
       <c r="D38" s="3"/>
       <c r="E38" s="1"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -1308,7 +1305,7 @@
       <c r="D39" s="3"/>
       <c r="E39" s="3"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -1319,7 +1316,7 @@
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -1330,8 +1327,8 @@
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" s="10" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="11" t="s">
         <v>4</v>
       </c>
       <c r="B42" s="6" t="s">
@@ -1347,8 +1344,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" s="11"/>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="12"/>
       <c r="B43" s="1">
         <f>COUNTIF(B2:B41, "Up")</f>
         <v>6</v>
@@ -1379,22 +1376,22 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21E34279-DF0B-49D0-978E-1339C67697A9}">
   <dimension ref="A1:I43"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="b">
+      <c r="C1" s="9" t="b">
         <v>0</v>
       </c>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1405,7 +1402,7 @@
       <c r="D2" s="7"/>
       <c r="E2" s="1"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1416,7 +1413,7 @@
       <c r="D3" s="7"/>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1427,7 +1424,7 @@
       <c r="D4" s="7"/>
       <c r="E4" s="7"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1438,7 +1435,7 @@
       <c r="D5" s="7"/>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1449,7 +1446,7 @@
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1460,7 +1457,7 @@
       <c r="D7" s="7"/>
       <c r="E7" s="7"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1471,7 +1468,7 @@
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1482,7 +1479,7 @@
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1493,7 +1490,7 @@
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1504,7 +1501,7 @@
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>11</v>
       </c>
@@ -1515,7 +1512,7 @@
       <c r="D12" s="7"/>
       <c r="E12" s="7"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>12</v>
       </c>
@@ -1525,11 +1522,11 @@
       <c r="C13" s="7"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="10"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>13</v>
       </c>
@@ -1540,7 +1537,7 @@
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>14</v>
       </c>
@@ -1551,7 +1548,7 @@
       <c r="D15" s="7"/>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>15</v>
       </c>
@@ -1562,7 +1559,7 @@
       <c r="D16" s="7"/>
       <c r="E16" s="1"/>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>16</v>
       </c>
@@ -1573,7 +1570,7 @@
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>17</v>
       </c>
@@ -1584,7 +1581,7 @@
       <c r="D18" s="7"/>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>18</v>
       </c>
@@ -1595,7 +1592,7 @@
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>19</v>
       </c>
@@ -1606,7 +1603,7 @@
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>20</v>
       </c>
@@ -1617,7 +1614,7 @@
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>21</v>
       </c>
@@ -1628,7 +1625,7 @@
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>22</v>
       </c>
@@ -1639,7 +1636,7 @@
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>23</v>
       </c>
@@ -1648,7 +1645,7 @@
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>24</v>
       </c>
@@ -1657,7 +1654,7 @@
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>25</v>
       </c>
@@ -1666,7 +1663,7 @@
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>26</v>
       </c>
@@ -1675,7 +1672,7 @@
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>27</v>
       </c>
@@ -1684,7 +1681,7 @@
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>28</v>
       </c>
@@ -1693,7 +1690,7 @@
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>29</v>
       </c>
@@ -1702,7 +1699,7 @@
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>30</v>
       </c>
@@ -1711,7 +1708,7 @@
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>31</v>
       </c>
@@ -1720,7 +1717,7 @@
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>32</v>
       </c>
@@ -1729,7 +1726,7 @@
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="1">
         <v>33</v>
       </c>
@@ -1738,7 +1735,7 @@
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="1">
         <v>34</v>
       </c>
@@ -1747,7 +1744,7 @@
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="1">
         <v>35</v>
       </c>
@@ -1756,7 +1753,7 @@
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="1">
         <v>36</v>
       </c>
@@ -1765,7 +1762,7 @@
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="1">
         <v>37</v>
       </c>
@@ -1774,7 +1771,7 @@
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="1">
         <v>38</v>
       </c>
@@ -1783,7 +1780,7 @@
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="1">
         <v>39</v>
       </c>
@@ -1792,7 +1789,7 @@
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -1801,8 +1798,8 @@
       <c r="D41" s="1"/>
       <c r="E41" s="1"/>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" s="10" t="s">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="11" t="s">
         <v>4</v>
       </c>
       <c r="B42" s="7" t="s">
@@ -1818,8 +1815,8 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" s="11"/>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="12"/>
       <c r="B43" s="1">
         <f>COUNTIF(B2:B41, "Up")</f>
         <v>6</v>
@@ -1850,15 +1847,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E66B4146-75A4-41C4-A73E-146E823D5C6D}">
   <dimension ref="A1:E41"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="5.875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3" style="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="5.88671875" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="13" t="s">
         <v>6</v>
       </c>
       <c r="B1" t="s">
@@ -1874,570 +1871,570 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="13">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="13">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="13">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="13">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="13">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="13">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="13">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D8" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="13">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="13">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="13">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C11" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="13">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D13" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="13">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D14" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="13">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C15" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="13">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D16" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="13">
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C17" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D17" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="13">
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C18" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D18" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="13">
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C19" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D19" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="13">
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C20" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D20" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="13">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D21" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="13">
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C22" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D22" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E22" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="13">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C23" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D23" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E23" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="13">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C24" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E24" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="13">
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C25" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D25" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E25" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="13">
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C26" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D26" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="13">
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C27" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D27" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="13">
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C28" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D28" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="13">
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C29" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="13">
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C30" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="14">
         <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="1">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="14">
         <v>31</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A33" s="1">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="14">
         <v>32</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A34" s="1">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="14">
         <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A35" s="1">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="14">
         <v>34</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A36" s="1">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="14">
         <v>35</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A37" s="1">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="14">
         <v>36</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A38" s="1">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="14">
         <v>37</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A39" s="1">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="14">
         <v>38</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A40" s="1">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="14">
         <v>39</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="12"/>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A41" s="1">
+      <c r="C40" s="8"/>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="14">
         <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
@@ -2453,7 +2450,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D72485C5-B1AA-46B0-AF62-B61CED32615E}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>